<commit_message>
Sync hardware deliverables and manual after pre-fab design review.
Refresh BOM (2026-07-09 CSV), Gerbers, EasyEDA project, pick-and-place, and schematic export; document corrected ADAU crystal/PLL strapping and Si4684 reference clock in the manual; add PCBWay acknowledgement on the back cover only.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Hardware/pic-and-place/PickAndPlace_PCB1_2026_07_05.xlsx
+++ b/Hardware/pic-and-place/PickAndPlace_PCB1_2026_07_05.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="PickAndPlace_PCB1_2026_07_05" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="PickAndPlace_PCB1_2026_07_09" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="417">
   <si>
     <t>Designator</t>
   </si>
@@ -958,12 +958,303 @@
     <t>10uF</t>
   </si>
   <si>
+    <t>U8</t>
+  </si>
+  <si>
+    <t>ESP32-S3-WROOM-1-N16</t>
+  </si>
+  <si>
+    <t>WIRELM-SMD_ESP32-S3-WROOM-1</t>
+  </si>
+  <si>
+    <t>73.279mm</t>
+  </si>
+  <si>
+    <t>38.862mm</t>
+  </si>
+  <si>
+    <t>64.529mm</t>
+  </si>
+  <si>
+    <t>47.757mm</t>
+  </si>
+  <si>
+    <t>2.4GHz</t>
+  </si>
+  <si>
+    <t>C33</t>
+  </si>
+  <si>
+    <t>48.641mm</t>
+  </si>
+  <si>
+    <t>22.352mm</t>
+  </si>
+  <si>
+    <t>49.641mm</t>
+  </si>
+  <si>
+    <t>C35</t>
+  </si>
+  <si>
+    <t>24.384mm</t>
+  </si>
+  <si>
+    <t>C40</t>
+  </si>
+  <si>
+    <t>48.387mm</t>
+  </si>
+  <si>
+    <t>17.923mm</t>
+  </si>
+  <si>
+    <t>C41</t>
+  </si>
+  <si>
+    <t>0402CG220J500NT</t>
+  </si>
+  <si>
+    <t>40.005mm</t>
+  </si>
+  <si>
+    <t>13.589mm</t>
+  </si>
+  <si>
+    <t>14.009mm</t>
+  </si>
+  <si>
+    <t>22pF</t>
+  </si>
+  <si>
+    <t>C43</t>
+  </si>
+  <si>
+    <t>31.393mm</t>
+  </si>
+  <si>
+    <t>23.689mm</t>
+  </si>
+  <si>
+    <t>24.689mm</t>
+  </si>
+  <si>
+    <t>C46</t>
+  </si>
+  <si>
+    <t>34.036mm</t>
+  </si>
+  <si>
+    <t>12.358mm</t>
+  </si>
+  <si>
+    <t>C47</t>
+  </si>
+  <si>
+    <t>32.258mm</t>
+  </si>
+  <si>
+    <t>18.796mm</t>
+  </si>
+  <si>
+    <t>19.796mm</t>
+  </si>
+  <si>
+    <t>R19</t>
+  </si>
+  <si>
+    <t>0402WGF2001TCE</t>
+  </si>
+  <si>
+    <t>30.48mm</t>
+  </si>
+  <si>
+    <t>20.447mm</t>
+  </si>
+  <si>
+    <t>20.88mm</t>
+  </si>
+  <si>
+    <t>2kΩ</t>
+  </si>
+  <si>
+    <t>C51</t>
+  </si>
+  <si>
+    <t>CC0603CPNPO9BN8R2</t>
+  </si>
+  <si>
+    <t>C0603</t>
+  </si>
+  <si>
+    <t>26.797mm</t>
+  </si>
+  <si>
+    <t>42.164mm</t>
+  </si>
+  <si>
+    <t>42.864mm</t>
+  </si>
+  <si>
+    <t>C52</t>
+  </si>
+  <si>
+    <t>0603B222K500NT</t>
+  </si>
+  <si>
+    <t>28.575mm</t>
+  </si>
+  <si>
+    <t>C53</t>
+  </si>
+  <si>
+    <t>CL10A105KB8NNNC</t>
+  </si>
+  <si>
+    <t>30.353mm</t>
+  </si>
+  <si>
+    <t>U11</t>
+  </si>
+  <si>
+    <t>FSC-BT1035</t>
+  </si>
+  <si>
+    <t>FSC-BT806</t>
+  </si>
+  <si>
+    <t>13.081mm</t>
+  </si>
+  <si>
+    <t>11.323mm</t>
+  </si>
+  <si>
+    <t>12.573mm</t>
+  </si>
+  <si>
+    <t>19.581mm</t>
+  </si>
+  <si>
+    <t>0.573mm</t>
+  </si>
+  <si>
+    <t>RF1</t>
+  </si>
+  <si>
+    <t>733910083</t>
+  </si>
+  <si>
+    <t>SMA-TH_733910083</t>
+  </si>
+  <si>
+    <t>4.064mm</t>
+  </si>
+  <si>
+    <t>6.604mm</t>
+  </si>
+  <si>
+    <t>40.259mm</t>
+  </si>
+  <si>
+    <t>18GHz</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>7.239mm</t>
+  </si>
+  <si>
+    <t>81.264mm</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>CL21A226MAQNNNE</t>
+  </si>
+  <si>
+    <t>83.693mm</t>
+  </si>
+  <si>
+    <t>16.891mm</t>
+  </si>
+  <si>
+    <t>82.693mm</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>80.153mm</t>
+  </si>
+  <si>
+    <t>18.018mm</t>
+  </si>
+  <si>
+    <t>19.018mm</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>59.563mm</t>
+  </si>
+  <si>
+    <t>46.228mm</t>
+  </si>
+  <si>
+    <t>58.563mm</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>60.348mm</t>
+  </si>
+  <si>
+    <t>60.781mm</t>
+  </si>
+  <si>
+    <t>R16</t>
+  </si>
+  <si>
+    <t>60.325mm</t>
+  </si>
+  <si>
+    <t>60.758mm</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>45.339mm</t>
+  </si>
+  <si>
+    <t>15.875mm</t>
+  </si>
+  <si>
+    <t>16.308mm</t>
+  </si>
+  <si>
+    <t>C49</t>
+  </si>
+  <si>
+    <t>0402CG150J500NT</t>
+  </si>
+  <si>
+    <t>19.812mm</t>
+  </si>
+  <si>
+    <t>15pF</t>
+  </si>
+  <si>
     <t>C50</t>
   </si>
   <si>
-    <t>0402CG120J500NT</t>
-  </si>
-  <si>
     <t>24.765mm</t>
   </si>
   <si>
@@ -971,285 +1262,6 @@
   </si>
   <si>
     <t>30.822mm</t>
-  </si>
-  <si>
-    <t>12pF</t>
-  </si>
-  <si>
-    <t>U8</t>
-  </si>
-  <si>
-    <t>ESP32-S3-WROOM-1-N16</t>
-  </si>
-  <si>
-    <t>WIRELM-SMD_ESP32-S3-WROOM-1</t>
-  </si>
-  <si>
-    <t>73.279mm</t>
-  </si>
-  <si>
-    <t>38.862mm</t>
-  </si>
-  <si>
-    <t>64.529mm</t>
-  </si>
-  <si>
-    <t>47.757mm</t>
-  </si>
-  <si>
-    <t>2.4GHz</t>
-  </si>
-  <si>
-    <t>C49</t>
-  </si>
-  <si>
-    <t>19.812mm</t>
-  </si>
-  <si>
-    <t>C33</t>
-  </si>
-  <si>
-    <t>48.641mm</t>
-  </si>
-  <si>
-    <t>22.352mm</t>
-  </si>
-  <si>
-    <t>49.641mm</t>
-  </si>
-  <si>
-    <t>C35</t>
-  </si>
-  <si>
-    <t>24.384mm</t>
-  </si>
-  <si>
-    <t>C40</t>
-  </si>
-  <si>
-    <t>48.387mm</t>
-  </si>
-  <si>
-    <t>17.923mm</t>
-  </si>
-  <si>
-    <t>C41</t>
-  </si>
-  <si>
-    <t>0402CG220J500NT</t>
-  </si>
-  <si>
-    <t>40.005mm</t>
-  </si>
-  <si>
-    <t>13.589mm</t>
-  </si>
-  <si>
-    <t>14.009mm</t>
-  </si>
-  <si>
-    <t>22pF</t>
-  </si>
-  <si>
-    <t>C43</t>
-  </si>
-  <si>
-    <t>31.393mm</t>
-  </si>
-  <si>
-    <t>23.689mm</t>
-  </si>
-  <si>
-    <t>24.689mm</t>
-  </si>
-  <si>
-    <t>C46</t>
-  </si>
-  <si>
-    <t>34.036mm</t>
-  </si>
-  <si>
-    <t>12.358mm</t>
-  </si>
-  <si>
-    <t>C47</t>
-  </si>
-  <si>
-    <t>32.258mm</t>
-  </si>
-  <si>
-    <t>18.796mm</t>
-  </si>
-  <si>
-    <t>19.796mm</t>
-  </si>
-  <si>
-    <t>R19</t>
-  </si>
-  <si>
-    <t>0402WGF2001TCE</t>
-  </si>
-  <si>
-    <t>30.48mm</t>
-  </si>
-  <si>
-    <t>20.447mm</t>
-  </si>
-  <si>
-    <t>20.88mm</t>
-  </si>
-  <si>
-    <t>2kΩ</t>
-  </si>
-  <si>
-    <t>C51</t>
-  </si>
-  <si>
-    <t>CC0603CPNPO9BN8R2</t>
-  </si>
-  <si>
-    <t>C0603</t>
-  </si>
-  <si>
-    <t>26.797mm</t>
-  </si>
-  <si>
-    <t>42.164mm</t>
-  </si>
-  <si>
-    <t>42.864mm</t>
-  </si>
-  <si>
-    <t>C52</t>
-  </si>
-  <si>
-    <t>0603B222K500NT</t>
-  </si>
-  <si>
-    <t>28.575mm</t>
-  </si>
-  <si>
-    <t>C53</t>
-  </si>
-  <si>
-    <t>CL10A105KB8NNNC</t>
-  </si>
-  <si>
-    <t>30.353mm</t>
-  </si>
-  <si>
-    <t>U11</t>
-  </si>
-  <si>
-    <t>FSC-BT1035</t>
-  </si>
-  <si>
-    <t>FSC-BT806</t>
-  </si>
-  <si>
-    <t>13.081mm</t>
-  </si>
-  <si>
-    <t>11.323mm</t>
-  </si>
-  <si>
-    <t>12.573mm</t>
-  </si>
-  <si>
-    <t>19.581mm</t>
-  </si>
-  <si>
-    <t>0.573mm</t>
-  </si>
-  <si>
-    <t>RF1</t>
-  </si>
-  <si>
-    <t>733910083</t>
-  </si>
-  <si>
-    <t>SMA-TH_733910083</t>
-  </si>
-  <si>
-    <t>4.064mm</t>
-  </si>
-  <si>
-    <t>6.604mm</t>
-  </si>
-  <si>
-    <t>40.259mm</t>
-  </si>
-  <si>
-    <t>18GHz</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>7.239mm</t>
-  </si>
-  <si>
-    <t>81.264mm</t>
-  </si>
-  <si>
-    <t>C4</t>
-  </si>
-  <si>
-    <t>CL21A226MAQNNNE</t>
-  </si>
-  <si>
-    <t>83.693mm</t>
-  </si>
-  <si>
-    <t>16.891mm</t>
-  </si>
-  <si>
-    <t>82.693mm</t>
-  </si>
-  <si>
-    <t>22uF</t>
-  </si>
-  <si>
-    <t>C5</t>
-  </si>
-  <si>
-    <t>80.153mm</t>
-  </si>
-  <si>
-    <t>18.018mm</t>
-  </si>
-  <si>
-    <t>19.018mm</t>
-  </si>
-  <si>
-    <t>C9</t>
-  </si>
-  <si>
-    <t>59.563mm</t>
-  </si>
-  <si>
-    <t>46.228mm</t>
-  </si>
-  <si>
-    <t>58.563mm</t>
-  </si>
-  <si>
-    <t>R1</t>
-  </si>
-  <si>
-    <t>60.348mm</t>
-  </si>
-  <si>
-    <t>60.781mm</t>
-  </si>
-  <si>
-    <t>R16</t>
-  </si>
-  <si>
-    <t>60.325mm</t>
-  </si>
-  <si>
-    <t>60.758mm</t>
   </si>
 </sst>
 </file>
@@ -1626,7 +1638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O85"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="15" width="20" customWidth="1"/>
@@ -4601,54 +4613,54 @@
         <v>316</v>
       </c>
       <c r="C64" t="s">
-        <v>40</v>
+        <v>317</v>
       </c>
       <c r="D64" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E64" t="s">
+        <v>319</v>
+      </c>
+      <c r="F64" t="s">
         <v>318</v>
       </c>
-      <c r="F64" t="s">
-        <v>317</v>
-      </c>
       <c r="G64" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H64" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="I64" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J64">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="K64" t="s">
         <v>22</v>
       </c>
       <c r="L64">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="M64" t="s">
         <v>23</v>
       </c>
       <c r="N64" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="O64" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B65" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="C65" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="D65" t="s">
         <v>324</v>
@@ -4666,54 +4678,54 @@
         <v>326</v>
       </c>
       <c r="I65" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J65">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="K65" t="s">
         <v>22</v>
       </c>
       <c r="L65">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="M65" t="s">
         <v>23</v>
       </c>
       <c r="N65" t="s">
-        <v>328</v>
+        <v>314</v>
       </c>
       <c r="O65" t="s">
-        <v>328</v>
+        <v>314</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B66" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C66" t="s">
-        <v>40</v>
+        <v>312</v>
       </c>
       <c r="D66" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="E66" t="s">
-        <v>205</v>
+        <v>328</v>
       </c>
       <c r="F66" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="G66" t="s">
-        <v>205</v>
+        <v>328</v>
       </c>
       <c r="H66" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="I66" t="s">
-        <v>206</v>
+        <v>328</v>
       </c>
       <c r="J66">
         <v>2</v>
@@ -4722,21 +4734,21 @@
         <v>22</v>
       </c>
       <c r="L66">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="M66" t="s">
         <v>23</v>
       </c>
       <c r="N66" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="O66" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B67" t="s">
         <v>311</v>
@@ -4745,22 +4757,22 @@
         <v>312</v>
       </c>
       <c r="D67" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E67" t="s">
-        <v>333</v>
+        <v>229</v>
       </c>
       <c r="F67" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G67" t="s">
-        <v>333</v>
+        <v>229</v>
       </c>
       <c r="H67" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="I67" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J67">
         <v>2</v>
@@ -4769,7 +4781,7 @@
         <v>22</v>
       </c>
       <c r="L67">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="M67" t="s">
         <v>23</v>
@@ -4783,25 +4795,25 @@
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>332</v>
+      </c>
+      <c r="B68" t="s">
+        <v>333</v>
+      </c>
+      <c r="C68" t="s">
+        <v>40</v>
+      </c>
+      <c r="D68" t="s">
+        <v>334</v>
+      </c>
+      <c r="E68" t="s">
         <v>335</v>
       </c>
-      <c r="B68" t="s">
-        <v>311</v>
-      </c>
-      <c r="C68" t="s">
-        <v>312</v>
-      </c>
-      <c r="D68" t="s">
-        <v>332</v>
-      </c>
-      <c r="E68" t="s">
-        <v>336</v>
-      </c>
       <c r="F68" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G68" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H68" t="s">
         <v>334</v>
@@ -4816,21 +4828,21 @@
         <v>22</v>
       </c>
       <c r="L68">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="M68" t="s">
         <v>23</v>
       </c>
       <c r="N68" t="s">
-        <v>314</v>
+        <v>337</v>
       </c>
       <c r="O68" t="s">
-        <v>314</v>
+        <v>337</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B69" t="s">
         <v>311</v>
@@ -4839,22 +4851,22 @@
         <v>312</v>
       </c>
       <c r="D69" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E69" t="s">
-        <v>229</v>
+        <v>340</v>
       </c>
       <c r="F69" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G69" t="s">
-        <v>229</v>
+        <v>340</v>
       </c>
       <c r="H69" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="I69" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="J69">
         <v>2</v>
@@ -4863,7 +4875,7 @@
         <v>22</v>
       </c>
       <c r="L69">
-        <v>90</v>
+        <v>270</v>
       </c>
       <c r="M69" t="s">
         <v>23</v>
@@ -4877,28 +4889,28 @@
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B70" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="C70" t="s">
         <v>40</v>
       </c>
       <c r="D70" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E70" t="s">
+        <v>298</v>
+      </c>
+      <c r="F70" t="s">
         <v>343</v>
       </c>
-      <c r="F70" t="s">
-        <v>342</v>
-      </c>
       <c r="G70" t="s">
+        <v>298</v>
+      </c>
+      <c r="H70" t="s">
         <v>343</v>
-      </c>
-      <c r="H70" t="s">
-        <v>342</v>
       </c>
       <c r="I70" t="s">
         <v>344</v>
@@ -4916,15 +4928,15 @@
         <v>23</v>
       </c>
       <c r="N70" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="O70" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B71" t="s">
         <v>311</v>
@@ -4933,22 +4945,22 @@
         <v>312</v>
       </c>
       <c r="D71" t="s">
+        <v>346</v>
+      </c>
+      <c r="E71" t="s">
         <v>347</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
+        <v>346</v>
+      </c>
+      <c r="G71" t="s">
+        <v>347</v>
+      </c>
+      <c r="H71" t="s">
+        <v>346</v>
+      </c>
+      <c r="I71" t="s">
         <v>348</v>
-      </c>
-      <c r="F71" t="s">
-        <v>347</v>
-      </c>
-      <c r="G71" t="s">
-        <v>348</v>
-      </c>
-      <c r="H71" t="s">
-        <v>347</v>
-      </c>
-      <c r="I71" t="s">
-        <v>349</v>
       </c>
       <c r="J71">
         <v>2</v>
@@ -4971,31 +4983,31 @@
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>349</v>
+      </c>
+      <c r="B72" t="s">
         <v>350</v>
       </c>
-      <c r="B72" t="s">
-        <v>341</v>
-      </c>
       <c r="C72" t="s">
-        <v>40</v>
+        <v>263</v>
       </c>
       <c r="D72" t="s">
         <v>351</v>
       </c>
       <c r="E72" t="s">
-        <v>298</v>
+        <v>352</v>
       </c>
       <c r="F72" t="s">
         <v>351</v>
       </c>
       <c r="G72" t="s">
-        <v>298</v>
+        <v>352</v>
       </c>
       <c r="H72" t="s">
         <v>351</v>
       </c>
       <c r="I72" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J72">
         <v>2</v>
@@ -5010,39 +5022,39 @@
         <v>23</v>
       </c>
       <c r="N72" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="O72" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B73" t="s">
-        <v>311</v>
+        <v>356</v>
       </c>
       <c r="C73" t="s">
-        <v>312</v>
+        <v>357</v>
       </c>
       <c r="D73" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="E73" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="F73" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="G73" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="H73" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="I73" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="J73">
         <v>2</v>
@@ -5057,39 +5069,39 @@
         <v>23</v>
       </c>
       <c r="N73" t="s">
-        <v>314</v>
+        <v>177</v>
       </c>
       <c r="O73" t="s">
-        <v>314</v>
+        <v>177</v>
       </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>361</v>
+      </c>
+      <c r="B74" t="s">
+        <v>362</v>
+      </c>
+      <c r="C74" t="s">
         <v>357</v>
       </c>
-      <c r="B74" t="s">
-        <v>358</v>
-      </c>
-      <c r="C74" t="s">
-        <v>263</v>
-      </c>
       <c r="D74" t="s">
+        <v>363</v>
+      </c>
+      <c r="E74" t="s">
         <v>359</v>
       </c>
-      <c r="E74" t="s">
+      <c r="F74" t="s">
+        <v>363</v>
+      </c>
+      <c r="G74" t="s">
+        <v>359</v>
+      </c>
+      <c r="H74" t="s">
+        <v>363</v>
+      </c>
+      <c r="I74" t="s">
         <v>360</v>
-      </c>
-      <c r="F74" t="s">
-        <v>359</v>
-      </c>
-      <c r="G74" t="s">
-        <v>360</v>
-      </c>
-      <c r="H74" t="s">
-        <v>359</v>
-      </c>
-      <c r="I74" t="s">
-        <v>361</v>
       </c>
       <c r="J74">
         <v>2</v>
@@ -5104,39 +5116,39 @@
         <v>23</v>
       </c>
       <c r="N74" t="s">
-        <v>362</v>
+        <v>306</v>
       </c>
       <c r="O74" t="s">
-        <v>362</v>
+        <v>306</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B75" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C75" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="D75" t="s">
         <v>366</v>
       </c>
       <c r="E75" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="F75" t="s">
         <v>366</v>
       </c>
       <c r="G75" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="H75" t="s">
         <v>366</v>
       </c>
       <c r="I75" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="J75">
         <v>2</v>
@@ -5151,136 +5163,136 @@
         <v>23</v>
       </c>
       <c r="N75" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="O75" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>367</v>
+      </c>
+      <c r="B76" t="s">
+        <v>368</v>
+      </c>
+      <c r="C76" t="s">
         <v>369</v>
       </c>
-      <c r="B76" t="s">
+      <c r="D76" t="s">
         <v>370</v>
       </c>
-      <c r="C76" t="s">
-        <v>365</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>371</v>
       </c>
-      <c r="E76" t="s">
-        <v>367</v>
-      </c>
       <c r="F76" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G76" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="H76" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="I76" t="s">
+        <v>374</v>
+      </c>
+      <c r="J76">
+        <v>52</v>
+      </c>
+      <c r="K76" t="s">
+        <v>22</v>
+      </c>
+      <c r="L76">
+        <v>180</v>
+      </c>
+      <c r="M76" t="s">
+        <v>23</v>
+      </c>
+      <c r="N76" t="s">
         <v>368</v>
       </c>
-      <c r="J76">
-        <v>2</v>
-      </c>
-      <c r="K76" t="s">
-        <v>22</v>
-      </c>
-      <c r="L76">
-        <v>270</v>
-      </c>
-      <c r="M76" t="s">
-        <v>23</v>
-      </c>
-      <c r="N76" t="s">
-        <v>306</v>
-      </c>
       <c r="O76" t="s">
-        <v>306</v>
+        <v>368</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B77" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C77" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="D77" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="E77" t="s">
-        <v>367</v>
+        <v>42</v>
       </c>
       <c r="F77" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="G77" t="s">
-        <v>367</v>
+        <v>42</v>
       </c>
       <c r="H77" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="I77" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="J77">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K77" t="s">
         <v>22</v>
       </c>
       <c r="L77">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="M77" t="s">
-        <v>23</v>
+        <v>122</v>
       </c>
       <c r="N77" t="s">
-        <v>167</v>
+        <v>381</v>
       </c>
       <c r="O77" t="s">
-        <v>167</v>
+        <v>381</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="B78" t="s">
-        <v>376</v>
+        <v>311</v>
       </c>
       <c r="C78" t="s">
-        <v>377</v>
+        <v>312</v>
       </c>
       <c r="D78" t="s">
-        <v>378</v>
+        <v>159</v>
       </c>
       <c r="E78" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="F78" t="s">
-        <v>378</v>
+        <v>159</v>
       </c>
       <c r="G78" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="H78" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="I78" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="J78">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="K78" t="s">
         <v>22</v>
@@ -5292,86 +5304,86 @@
         <v>23</v>
       </c>
       <c r="N78" t="s">
-        <v>376</v>
+        <v>314</v>
       </c>
       <c r="O78" t="s">
-        <v>376</v>
+        <v>314</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B79" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C79" t="s">
-        <v>385</v>
+        <v>312</v>
       </c>
       <c r="D79" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E79" t="s">
-        <v>42</v>
+        <v>388</v>
       </c>
       <c r="F79" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G79" t="s">
-        <v>42</v>
+        <v>388</v>
       </c>
       <c r="H79" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="I79" t="s">
         <v>388</v>
       </c>
       <c r="J79">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K79" t="s">
         <v>22</v>
       </c>
       <c r="L79">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="M79" t="s">
-        <v>122</v>
+        <v>23</v>
       </c>
       <c r="N79" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="O79" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B80" t="s">
-        <v>311</v>
+        <v>386</v>
       </c>
       <c r="C80" t="s">
         <v>312</v>
       </c>
       <c r="D80" t="s">
-        <v>159</v>
+        <v>392</v>
       </c>
       <c r="E80" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F80" t="s">
-        <v>159</v>
+        <v>392</v>
       </c>
       <c r="G80" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="H80" t="s">
         <v>392</v>
       </c>
       <c r="I80" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="J80">
         <v>2</v>
@@ -5380,45 +5392,45 @@
         <v>22</v>
       </c>
       <c r="L80">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="M80" t="s">
         <v>23</v>
       </c>
       <c r="N80" t="s">
-        <v>314</v>
+        <v>390</v>
       </c>
       <c r="O80" t="s">
-        <v>314</v>
+        <v>390</v>
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B81" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="C81" t="s">
         <v>312</v>
       </c>
       <c r="D81" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E81" t="s">
+        <v>397</v>
+      </c>
+      <c r="F81" t="s">
         <v>396</v>
       </c>
-      <c r="F81" t="s">
-        <v>395</v>
-      </c>
       <c r="G81" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="H81" t="s">
+        <v>398</v>
+      </c>
+      <c r="I81" t="s">
         <v>397</v>
-      </c>
-      <c r="I81" t="s">
-        <v>396</v>
       </c>
       <c r="J81">
         <v>2</v>
@@ -5433,10 +5445,10 @@
         <v>23</v>
       </c>
       <c r="N81" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="O81" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
@@ -5444,28 +5456,28 @@
         <v>399</v>
       </c>
       <c r="B82" t="s">
-        <v>394</v>
+        <v>350</v>
       </c>
       <c r="C82" t="s">
-        <v>312</v>
+        <v>263</v>
       </c>
       <c r="D82" t="s">
         <v>400</v>
       </c>
       <c r="E82" t="s">
-        <v>401</v>
+        <v>220</v>
       </c>
       <c r="F82" t="s">
         <v>400</v>
       </c>
       <c r="G82" t="s">
+        <v>220</v>
+      </c>
+      <c r="H82" t="s">
         <v>401</v>
       </c>
-      <c r="H82" t="s">
-        <v>400</v>
-      </c>
       <c r="I82" t="s">
-        <v>402</v>
+        <v>220</v>
       </c>
       <c r="J82">
         <v>2</v>
@@ -5474,45 +5486,45 @@
         <v>22</v>
       </c>
       <c r="L82">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="M82" t="s">
         <v>23</v>
       </c>
       <c r="N82" t="s">
-        <v>398</v>
+        <v>354</v>
       </c>
       <c r="O82" t="s">
-        <v>398</v>
+        <v>354</v>
       </c>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>402</v>
+      </c>
+      <c r="B83" t="s">
+        <v>350</v>
+      </c>
+      <c r="C83" t="s">
+        <v>263</v>
+      </c>
+      <c r="D83" t="s">
         <v>403</v>
       </c>
-      <c r="B83" t="s">
-        <v>394</v>
-      </c>
-      <c r="C83" t="s">
-        <v>312</v>
-      </c>
-      <c r="D83" t="s">
+      <c r="E83" t="s">
+        <v>274</v>
+      </c>
+      <c r="F83" t="s">
+        <v>403</v>
+      </c>
+      <c r="G83" t="s">
+        <v>274</v>
+      </c>
+      <c r="H83" t="s">
         <v>404</v>
       </c>
-      <c r="E83" t="s">
-        <v>405</v>
-      </c>
-      <c r="F83" t="s">
-        <v>404</v>
-      </c>
-      <c r="G83" t="s">
-        <v>405</v>
-      </c>
-      <c r="H83" t="s">
-        <v>406</v>
-      </c>
       <c r="I83" t="s">
-        <v>405</v>
+        <v>274</v>
       </c>
       <c r="J83">
         <v>2</v>
@@ -5521,46 +5533,46 @@
         <v>22</v>
       </c>
       <c r="L83">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="M83" t="s">
         <v>23</v>
       </c>
       <c r="N83" t="s">
-        <v>398</v>
+        <v>354</v>
       </c>
       <c r="O83" t="s">
-        <v>398</v>
+        <v>354</v>
       </c>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B84" t="s">
-        <v>358</v>
+        <v>269</v>
       </c>
       <c r="C84" t="s">
         <v>263</v>
       </c>
       <c r="D84" t="s">
+        <v>406</v>
+      </c>
+      <c r="E84" t="s">
+        <v>407</v>
+      </c>
+      <c r="F84" t="s">
+        <v>406</v>
+      </c>
+      <c r="G84" t="s">
+        <v>407</v>
+      </c>
+      <c r="H84" t="s">
+        <v>406</v>
+      </c>
+      <c r="I84" t="s">
         <v>408</v>
       </c>
-      <c r="E84" t="s">
-        <v>220</v>
-      </c>
-      <c r="F84" t="s">
-        <v>408</v>
-      </c>
-      <c r="G84" t="s">
-        <v>220</v>
-      </c>
-      <c r="H84" t="s">
-        <v>409</v>
-      </c>
-      <c r="I84" t="s">
-        <v>220</v>
-      </c>
       <c r="J84">
         <v>2</v>
       </c>
@@ -5568,63 +5580,110 @@
         <v>22</v>
       </c>
       <c r="L84">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="M84" t="s">
         <v>23</v>
       </c>
       <c r="N84" t="s">
-        <v>362</v>
+        <v>271</v>
       </c>
       <c r="O84" t="s">
-        <v>362</v>
+        <v>271</v>
       </c>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>409</v>
+      </c>
+      <c r="B85" t="s">
         <v>410</v>
       </c>
-      <c r="B85" t="s">
-        <v>358</v>
-      </c>
       <c r="C85" t="s">
-        <v>263</v>
+        <v>40</v>
       </c>
       <c r="D85" t="s">
         <v>411</v>
       </c>
       <c r="E85" t="s">
-        <v>274</v>
+        <v>205</v>
       </c>
       <c r="F85" t="s">
         <v>411</v>
       </c>
       <c r="G85" t="s">
-        <v>274</v>
+        <v>205</v>
       </c>
       <c r="H85" t="s">
+        <v>411</v>
+      </c>
+      <c r="I85" t="s">
+        <v>206</v>
+      </c>
+      <c r="J85">
+        <v>2</v>
+      </c>
+      <c r="K85" t="s">
+        <v>22</v>
+      </c>
+      <c r="L85">
+        <v>90</v>
+      </c>
+      <c r="M85" t="s">
+        <v>23</v>
+      </c>
+      <c r="N85" t="s">
         <v>412</v>
       </c>
-      <c r="I85" t="s">
-        <v>274</v>
-      </c>
-      <c r="J85">
-        <v>2</v>
-      </c>
-      <c r="K85" t="s">
-        <v>22</v>
-      </c>
-      <c r="L85">
-        <v>180</v>
-      </c>
-      <c r="M85" t="s">
-        <v>23</v>
-      </c>
-      <c r="N85" t="s">
-        <v>362</v>
-      </c>
       <c r="O85" t="s">
-        <v>362</v>
+        <v>412</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>413</v>
+      </c>
+      <c r="B86" t="s">
+        <v>410</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86" t="s">
+        <v>414</v>
+      </c>
+      <c r="E86" t="s">
+        <v>415</v>
+      </c>
+      <c r="F86" t="s">
+        <v>414</v>
+      </c>
+      <c r="G86" t="s">
+        <v>415</v>
+      </c>
+      <c r="H86" t="s">
+        <v>414</v>
+      </c>
+      <c r="I86" t="s">
+        <v>416</v>
+      </c>
+      <c r="J86">
+        <v>2</v>
+      </c>
+      <c r="K86" t="s">
+        <v>22</v>
+      </c>
+      <c r="L86">
+        <v>90</v>
+      </c>
+      <c r="M86" t="s">
+        <v>23</v>
+      </c>
+      <c r="N86" t="s">
+        <v>412</v>
+      </c>
+      <c r="O86" t="s">
+        <v>412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>